<commit_message>
fix: corrige resultados ND e fontes da extração
</commit_message>
<xml_diff>
--- a/data/modelos/mapa_extracao.xlsx
+++ b/data/modelos/mapa_extracao.xlsx
@@ -7,7 +7,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extração" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -825,7 +825,7 @@
     <row r="11">
       <c r="A11" s="24" t="inlineStr">
         <is>
-          <t>Preencher o nome do ensaio com o padrão DENVDDMMAA-N (em que N é o número da placa de extração do dia).</t>
+          <t>Preencher o nome do ensaio com o padrão HPVDDMMAA# (em que # é o número da placa de extração do dia).</t>
         </is>
       </c>
       <c r="B11" s="22" t="n"/>
@@ -940,9 +940,33 @@
       <c r="L1" s="50" t="n"/>
       <c r="M1" s="54" t="inlineStr">
         <is>
-          <t>REVISÃO
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>REVISÃO</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t xml:space="preserve">
 00
-Página 1 de 1</t>
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <color theme="1"/>
+              <sz val="7"/>
+            </rPr>
+            <t>Página 1 de 1</t>
+          </r>
         </is>
       </c>
       <c r="N1" s="52" t="n"/>
@@ -952,9 +976,43 @@
       <c r="C2" s="56" t="n"/>
       <c r="D2" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">FORMULÁRIO
-LACEN/CEVS
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>FORMULÁRIO</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="8"/>
+            </rPr>
+            <t>
 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="10"/>
+            </rPr>
+            <t>LACEN/CEVS</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial, sans-serif"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="12"/>
+            </rPr>
+            <t>
+</t>
+          </r>
         </is>
       </c>
       <c r="E2" s="49" t="n"/>
@@ -1000,13 +1058,13 @@
         </is>
       </c>
       <c r="L4" s="25">
-        <f>"Ensaio: "&amp;Amostras!B1</f>
+        <f>concat("Ensaio: ",Amostras!B1)</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="25.5" customHeight="1" s="47">
-      <c r="A5" s="29" t="n"/>
-      <c r="B5" s="30" t="n"/>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="27" t="n"/>
       <c r="C5" s="28" t="n">
         <v>1</v>
       </c>

</xml_diff>